<commit_message>
final version of the repo hopefully
</commit_message>
<xml_diff>
--- a/Code/df.xlsx
+++ b/Code/df.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matyasvarga-etele/Desktop/Projects/Project-Financial-Instruments-Paper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matyasvarga-etele/Desktop/Projects/Project-Financial-Instruments-Paper/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FBCFEB-AF84-A740-BCA4-7D1AF0E0D5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD2BA9B-EDF0-2C41-B65A-924C2029AE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48160" yWindow="-2320" windowWidth="16520" windowHeight="15820" xr2:uid="{A073BFCF-4CB7-1949-B863-6AEAFEE7C6B0}"/>
+    <workbookView xWindow="29900" yWindow="-20" windowWidth="16520" windowHeight="15820" xr2:uid="{A073BFCF-4CB7-1949-B863-6AEAFEE7C6B0}"/>
   </bookViews>
   <sheets>
     <sheet name="df" sheetId="1" r:id="rId1"/>
@@ -292,8 +292,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -371,7 +371,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -381,13 +381,13 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>